<commit_message>
Improve S00026 PASS rate: 29→30 (session 11)
- Generalize annuity formula extraction with min_entry_age parsing:
  extract '가입최저나이 : [만 ]N세' from text (default 0)
- Fixes 1772 (e연금저축보험): min_age=19 instead of 0
- Resolves structural_issues.xlsx items 1224, 1228 → '해결'
- Update docs/작업일지.md with session 11 progress

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/structural_issues.xlsx
+++ b/data/structural_issues.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="77295" yWindow="150" windowWidth="26010" windowHeight="10545" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="구조적 문제" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -19,29 +18,42 @@
   <numFmts count="0"/>
   <fonts count="5">
     <font>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
       <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="000563C1"/>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
+      <color rgb="FF0563C1"/>
       <sz val="10"/>
       <u val="single"/>
     </font>
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
       <i val="1"/>
-      <color rgb="00595959"/>
+      <color rgb="FF595959"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
+      <sz val="8"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -53,24 +65,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
+        <fgColor rgb="FF1F4E79"/>
+        <bgColor rgb="FF1F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-        <bgColor rgb="00FFEB9C"/>
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -79,24 +91,19 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
-    <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -104,33 +111,33 @@
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -494,7 +501,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F67"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>
@@ -557,10 +564,14 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr"/>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">보기납기 조합이 하나일 경우는 가입나이테이블에 보기납기 정보가 필요없음. </t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="2" t="n">
@@ -583,16 +594,23 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr"/>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>나.보험료 납입기간 항목이 납입기간 정보 이다.
+(2) 가입최고나이 : (연금개시나이-납입기간)세  계산하고
+마. 연금개시나이 - 만 55세~80세  정보가 있다. 
+이련 형태도 일반화 하여 추출 가능하도록 해줘</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>1550</v>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
+      <c r="B4" s="5" t="n"/>
       <c r="C4" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -608,13 +626,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="n"/>
     </row>
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>1555</v>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
+      <c r="B5" s="5" t="n"/>
       <c r="C5" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -630,7 +648,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="n"/>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="6" t="n">
@@ -656,7 +674,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>2. 보험기간, 보험료 납입기간, 보험료 납입주기, 피보험자 가입나이 및 연금개시나이 : 보험기간 납입기간 납입주기 연금개시나이 정보가 있는 부분이다.
+나.  보험종목의 구성 이  동일한 ISRN_KIND_DTCD의 ITCD 구분 정보이다. 이 정보를 활용하여 구분 해야 한다.
+이런형태의 서류가 몇개더 있어 그래서 일반화 하여 다른 사업방법서 추출할때도 사용가능하도록 해주라.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -682,13 +706,19 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr"/>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>2. 보험기간, 보험료 납입기간, 보험료 납입주기, 피보험자 가입나이 및 연금개시나이 : 보험기간 납입기간 납입주기 연금개시나이 정보가 있는 부분이다.
+나.  보험종목의 구성 이  동일한 ISRN_KIND_DTCD의 ITCD 구분 정보이다. 이 정보를 활용하여 구분 해야 한다.
+이런형태의 서류가 몇개더 있어 그래서 일반화 하여 다른 사업방법서 추출할때도 사용가능하도록 해주라.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>1626</v>
       </c>
-      <c r="B8" s="5" t="inlineStr"/>
+      <c r="B8" s="5" t="n"/>
       <c r="C8" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -704,7 +734,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr"/>
+      <c r="F8" s="4" t="n"/>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="2" t="n">
@@ -730,7 +760,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr"/>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>2. 보험기간, 보험료 납입기간, 보험료 납입주기, 피보험자 가입나이 및 연금개시나이 : 보험기간 납입기간 납입주기 연금개시나이 정보가 있는 부분이다.
+나.  보험종목의 구성 이  동일한 ISRN_KIND_DTCD의 ITCD 구분 정보이다. 이 정보를 활용하여 구분 해야 한다.
+이런형태의 서류가 몇개더 있어 그래서 일반화 하여 다른 사업방법서 추출할때도 사용가능하도록 해주라.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -756,13 +792,19 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr"/>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>2. 보험기간, 보험료 납입기간, 보험료 납입주기, 피보험자 가입나이 및 연금개시나이 : 보험기간 납입기간 납입주기 연금개시나이 정보가 있는 부분이다.
+나.  보험종목의 구성 이  동일한 ISRN_KIND_DTCD의 ITCD 구분 정보이다. 이 정보를 활용하여 구분 해야 한다.
+이런형태의 서류가 몇개더 있어 그래서 일반화 하여 다른 사업방법서 추출할때도 사용가능하도록 해주라.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>1651</v>
       </c>
-      <c r="B11" s="5" t="inlineStr"/>
+      <c r="B11" s="5" t="n"/>
       <c r="C11" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -778,13 +820,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="n"/>
     </row>
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>1671</v>
       </c>
-      <c r="B12" s="5" t="inlineStr"/>
+      <c r="B12" s="5" t="n"/>
       <c r="C12" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -800,13 +842,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr"/>
+      <c r="F12" s="4" t="n"/>
     </row>
     <row r="13" ht="36" customHeight="1">
       <c r="A13" s="2" t="n">
         <v>1700</v>
       </c>
-      <c r="B13" s="5" t="inlineStr"/>
+      <c r="B13" s="5" t="n"/>
       <c r="C13" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -822,13 +864,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr"/>
+      <c r="F13" s="4" t="n"/>
     </row>
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>1708</v>
       </c>
-      <c r="B14" s="5" t="inlineStr"/>
+      <c r="B14" s="5" t="n"/>
       <c r="C14" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -844,13 +886,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="n"/>
     </row>
     <row r="15" ht="36" customHeight="1">
       <c r="A15" s="2" t="n">
         <v>1709</v>
       </c>
-      <c r="B15" s="5" t="inlineStr"/>
+      <c r="B15" s="5" t="n"/>
       <c r="C15" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -866,7 +908,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr"/>
+      <c r="F15" s="4" t="n"/>
     </row>
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -892,13 +934,17 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr"/>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>만19세를 19세 인식하게 해줘</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="2" t="n">
         <v>1736</v>
       </c>
-      <c r="B17" s="5" t="inlineStr"/>
+      <c r="B17" s="5" t="n"/>
       <c r="C17" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -914,13 +960,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="n"/>
     </row>
     <row r="18" ht="36" customHeight="1">
       <c r="A18" s="2" t="n">
         <v>1743</v>
       </c>
-      <c r="B18" s="5" t="inlineStr"/>
+      <c r="B18" s="5" t="n"/>
       <c r="C18" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -936,7 +982,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="n"/>
     </row>
     <row r="19" ht="36" customHeight="1">
       <c r="A19" s="2" t="n">
@@ -962,7 +1008,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr"/>
+      <c r="F19" s="4" t="n"/>
     </row>
     <row r="20" ht="36" customHeight="1">
       <c r="A20" s="6" t="n">
@@ -988,13 +1034,19 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr"/>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>1. 보험종목에 관한 사항
+나.  보험종목의 구성 이  동일한 ISRN_KIND_DTCD의 ITCD 구분 정보이다. 이 정보를 활용하여 구분 해야 한다.
+이런형태의 서류가 몇개더 있어 그래서 일반화 하여 다른 사업방법서 추출할때도 사용가능하도록 해주라.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="36" customHeight="1">
       <c r="A21" s="2" t="n">
         <v>1752</v>
       </c>
-      <c r="B21" s="5" t="inlineStr"/>
+      <c r="B21" s="5" t="n"/>
       <c r="C21" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -1010,13 +1062,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="n"/>
     </row>
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="2" t="n">
         <v>1753</v>
       </c>
-      <c r="B22" s="5" t="inlineStr"/>
+      <c r="B22" s="5" t="n"/>
       <c r="C22" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -1032,7 +1084,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr"/>
+      <c r="F22" s="4" t="n"/>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="2" t="n">
@@ -1058,13 +1110,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="n"/>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="2" t="n">
         <v>1760</v>
       </c>
-      <c r="B24" s="5" t="inlineStr"/>
+      <c r="B24" s="5" t="n"/>
       <c r="C24" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -1080,7 +1132,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr"/>
+      <c r="F24" s="4" t="n"/>
     </row>
     <row r="25" ht="36" customHeight="1">
       <c r="A25" s="2" t="n">
@@ -1106,7 +1158,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="n"/>
     </row>
     <row r="26" ht="36" customHeight="1">
       <c r="A26" s="2" t="n">
@@ -1132,13 +1184,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="n"/>
     </row>
     <row r="27" ht="36" customHeight="1">
       <c r="A27" s="2" t="n">
         <v>1781</v>
       </c>
-      <c r="B27" s="5" t="inlineStr"/>
+      <c r="B27" s="5" t="n"/>
       <c r="C27" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -1154,13 +1206,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="n"/>
     </row>
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="2" t="n">
         <v>1789</v>
       </c>
-      <c r="B28" s="5" t="inlineStr"/>
+      <c r="B28" s="5" t="n"/>
       <c r="C28" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -1176,13 +1228,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr"/>
+      <c r="F28" s="4" t="n"/>
     </row>
     <row r="29" ht="36" customHeight="1">
       <c r="A29" s="2" t="n">
         <v>1795</v>
       </c>
-      <c r="B29" s="5" t="inlineStr"/>
+      <c r="B29" s="5" t="n"/>
       <c r="C29" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -1198,7 +1250,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr"/>
+      <c r="F29" s="4" t="n"/>
     </row>
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="2" t="n">
@@ -1224,7 +1276,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr"/>
+      <c r="F30" s="4" t="n"/>
     </row>
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="2" t="n">
@@ -1250,7 +1302,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="n"/>
     </row>
     <row r="32" ht="36" customHeight="1">
       <c r="A32" s="2" t="n">
@@ -1276,13 +1328,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr"/>
+      <c r="F32" s="4" t="n"/>
     </row>
     <row r="33" ht="36" customHeight="1">
       <c r="A33" s="2" t="n">
         <v>1845</v>
       </c>
-      <c r="B33" s="5" t="inlineStr"/>
+      <c r="B33" s="5" t="n"/>
       <c r="C33" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -1298,7 +1350,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr"/>
+      <c r="F33" s="4" t="n"/>
     </row>
     <row r="34" ht="36" customHeight="1">
       <c r="A34" s="2" t="n">
@@ -1324,7 +1376,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr"/>
+      <c r="F34" s="4" t="n"/>
     </row>
     <row r="35" ht="36" customHeight="1">
       <c r="A35" s="2" t="n">
@@ -1350,7 +1402,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr"/>
+      <c r="F35" s="4" t="n"/>
     </row>
     <row r="36" ht="36" customHeight="1">
       <c r="A36" s="2" t="n">
@@ -1376,7 +1428,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="n"/>
     </row>
     <row r="37" ht="36" customHeight="1">
       <c r="A37" s="2" t="n">
@@ -1402,7 +1454,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="n"/>
     </row>
     <row r="38" ht="36" customHeight="1">
       <c r="A38" s="2" t="n">
@@ -1428,7 +1480,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr"/>
+      <c r="F38" s="4" t="n"/>
     </row>
     <row r="39" ht="36" customHeight="1">
       <c r="A39" s="2" t="n">
@@ -1454,7 +1506,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr"/>
+      <c r="F39" s="4" t="n"/>
     </row>
     <row r="40" ht="36" customHeight="1">
       <c r="A40" s="2" t="n">
@@ -1480,7 +1532,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr"/>
+      <c r="F40" s="4" t="n"/>
     </row>
     <row r="41" ht="36" customHeight="1">
       <c r="A41" s="2" t="n">
@@ -1506,7 +1558,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="n"/>
     </row>
     <row r="42" ht="36" customHeight="1">
       <c r="A42" s="2" t="n">
@@ -1532,7 +1584,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F42" s="4" t="inlineStr"/>
+      <c r="F42" s="4" t="n"/>
     </row>
     <row r="43" ht="36" customHeight="1">
       <c r="A43" s="2" t="n">
@@ -1558,13 +1610,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="n"/>
     </row>
     <row r="44" ht="36" customHeight="1">
       <c r="A44" s="2" t="n">
         <v>2127</v>
       </c>
-      <c r="B44" s="5" t="inlineStr"/>
+      <c r="B44" s="5" t="n"/>
       <c r="C44" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -1580,13 +1632,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr"/>
+      <c r="F44" s="4" t="n"/>
     </row>
     <row r="45" ht="36" customHeight="1">
       <c r="A45" s="2" t="n">
         <v>2128</v>
       </c>
-      <c r="B45" s="5" t="inlineStr"/>
+      <c r="B45" s="5" t="n"/>
       <c r="C45" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -1602,7 +1654,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="n"/>
     </row>
     <row r="46" ht="36" customHeight="1">
       <c r="A46" s="2" t="n">
@@ -1628,7 +1680,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr"/>
+      <c r="F46" s="4" t="n"/>
     </row>
     <row r="47" ht="36" customHeight="1">
       <c r="A47" s="2" t="n">
@@ -1654,7 +1706,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F47" s="4" t="inlineStr"/>
+      <c r="F47" s="4" t="n"/>
     </row>
     <row r="48" ht="36" customHeight="1">
       <c r="A48" s="6" t="n">
@@ -1680,13 +1732,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F48" s="8" t="inlineStr"/>
+      <c r="F48" s="8" t="n"/>
     </row>
     <row r="49" ht="36" customHeight="1">
       <c r="A49" s="2" t="n">
         <v>2172</v>
       </c>
-      <c r="B49" s="5" t="inlineStr"/>
+      <c r="B49" s="5" t="n"/>
       <c r="C49" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -1702,13 +1754,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F49" s="4" t="inlineStr"/>
+      <c r="F49" s="4" t="n"/>
     </row>
     <row r="50" ht="36" customHeight="1">
       <c r="A50" s="2" t="n">
         <v>2174</v>
       </c>
-      <c r="B50" s="5" t="inlineStr"/>
+      <c r="B50" s="5" t="n"/>
       <c r="C50" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -1724,7 +1776,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr"/>
+      <c r="F50" s="4" t="n"/>
     </row>
     <row r="51" ht="36" customHeight="1">
       <c r="A51" s="6" t="n">
@@ -1750,7 +1802,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F51" s="8" t="inlineStr"/>
+      <c r="F51" s="8" t="n"/>
     </row>
     <row r="52" ht="36" customHeight="1">
       <c r="A52" s="2" t="n">
@@ -1776,7 +1828,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F52" s="4" t="inlineStr"/>
+      <c r="F52" s="4" t="n"/>
     </row>
     <row r="53" ht="36" customHeight="1">
       <c r="A53" s="2" t="n">
@@ -1802,7 +1854,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F53" s="4" t="inlineStr"/>
+      <c r="F53" s="4" t="n"/>
     </row>
     <row r="54" ht="36" customHeight="1">
       <c r="A54" s="2" t="n">
@@ -1828,7 +1880,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F54" s="4" t="inlineStr"/>
+      <c r="F54" s="4" t="n"/>
     </row>
     <row r="55" ht="36" customHeight="1">
       <c r="A55" s="2" t="n">
@@ -1854,7 +1906,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F55" s="4" t="inlineStr"/>
+      <c r="F55" s="4" t="n"/>
     </row>
     <row r="56" ht="36" customHeight="1">
       <c r="A56" s="2" t="n">
@@ -1880,7 +1932,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr"/>
+      <c r="F56" s="4" t="n"/>
     </row>
     <row r="57" ht="36" customHeight="1">
       <c r="A57" s="2" t="n">
@@ -1906,7 +1958,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr"/>
+      <c r="F57" s="4" t="n"/>
     </row>
     <row r="58" ht="36" customHeight="1">
       <c r="A58" s="2" t="n">
@@ -1932,13 +1984,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F58" s="4" t="inlineStr"/>
+      <c r="F58" s="4" t="n"/>
     </row>
     <row r="59" ht="36" customHeight="1">
       <c r="A59" s="2" t="n">
         <v>2245</v>
       </c>
-      <c r="B59" s="5" t="inlineStr"/>
+      <c r="B59" s="5" t="n"/>
       <c r="C59" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -1954,7 +2006,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F59" s="4" t="inlineStr"/>
+      <c r="F59" s="4" t="n"/>
     </row>
     <row r="60" ht="36" customHeight="1">
       <c r="A60" s="2" t="n">
@@ -1980,13 +2032,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F60" s="4" t="inlineStr"/>
+      <c r="F60" s="4" t="n"/>
     </row>
     <row r="61" ht="36" customHeight="1">
       <c r="A61" s="2" t="n">
         <v>2247</v>
       </c>
-      <c r="B61" s="5" t="inlineStr"/>
+      <c r="B61" s="5" t="n"/>
       <c r="C61" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -2002,7 +2054,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F61" s="4" t="inlineStr"/>
+      <c r="F61" s="4" t="n"/>
     </row>
     <row r="62" ht="36" customHeight="1">
       <c r="A62" s="2" t="n">
@@ -2028,7 +2080,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F62" s="4" t="inlineStr"/>
+      <c r="F62" s="4" t="n"/>
     </row>
     <row r="63" ht="36" customHeight="1">
       <c r="A63" s="2" t="n">
@@ -2054,13 +2106,13 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F63" s="4" t="inlineStr"/>
+      <c r="F63" s="4" t="n"/>
     </row>
     <row r="64" ht="36" customHeight="1">
       <c r="A64" s="2" t="n">
         <v>2252</v>
       </c>
-      <c r="B64" s="5" t="inlineStr"/>
+      <c r="B64" s="5" t="n"/>
       <c r="C64" s="4" t="inlineStr">
         <is>
           <t>GT_NaN</t>
@@ -2076,7 +2128,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F64" s="4" t="inlineStr"/>
+      <c r="F64" s="4" t="n"/>
     </row>
     <row r="65" ht="36" customHeight="1">
       <c r="A65" s="2" t="n">
@@ -2102,7 +2154,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F65" s="4" t="inlineStr"/>
+      <c r="F65" s="4" t="n"/>
     </row>
     <row r="66" ht="36" customHeight="1">
       <c r="A66" s="2" t="n">
@@ -2128,7 +2180,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F66" s="4" t="inlineStr"/>
+      <c r="F66" s="4" t="n"/>
     </row>
     <row r="67" ht="36" customHeight="1">
       <c r="A67" s="2" t="n">
@@ -2154,7 +2206,7 @@
           <t>미해결</t>
         </is>
       </c>
-      <c r="F67" s="4" t="inlineStr"/>
+      <c r="F67" s="4" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2202,5 +2254,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B67" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add session-end structural analysis procedure and update status (session 12)
- Add scripts/update_structural_issues.py: auto-updates data/structural_issues.xlsx
  status (해결/미해결/처리불가) based on latest S00026 PASS/FAIL report
- Add session-end procedure section to CLAUDE.md (batch_run → generate_report → update_structural_issues)
- Update structural_issues.xlsx: 16 rows updated (1571/1629/1726/1745/2130/2205 → 처리불가, 1808/1946/1950/1976/1985/1986/2244/2246/2255/2256 → 해결, 1629/1772 → 해결)
- Refresh extracted outputs and reports (batch rerun confirming PASS=30)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/structural_issues.xlsx
+++ b/data/structural_issues.xlsx
@@ -56,7 +56,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -79,6 +79,21 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
         <bgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -109,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -133,6 +148,15 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -562,7 +586,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>해결</t>
         </is>
@@ -592,7 +616,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>해결</t>
         </is>
@@ -669,9 +693,9 @@
           <t>동일 PDF 내 복수 ITCD 간 보험기간/납입기간 상이</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>처리불가</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -701,7 +725,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -755,9 +779,9 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -787,9 +811,9 @@
           <t>동일 PDF 내 복수 ITCD 간 보험기간/납입기간 상이</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -929,9 +953,9 @@
           <t>ITCD 039/041 MIN_AG=19, ITCD 040/042 MIN_AG=20 — PDF에 만19세만 존재</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>처리불가</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -1003,7 +1027,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1029,9 +1053,9 @@
           <t>동일 PDF 내 복수 ITCD 간 MIN_AG 상이</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>처리불가</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -1105,7 +1129,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1153,7 +1177,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1179,9 +1203,9 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F26" s="4" t="n"/>
@@ -1271,9 +1295,9 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F30" s="4" t="n"/>
@@ -1297,7 +1321,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="E31" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1323,7 +1347,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1371,9 +1395,9 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F34" s="4" t="n"/>
@@ -1397,9 +1421,9 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F35" s="4" t="n"/>
@@ -1423,9 +1447,9 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F36" s="4" t="n"/>
@@ -1449,7 +1473,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E37" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1475,7 +1499,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1501,7 +1525,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E39" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1527,9 +1551,9 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F40" s="4" t="n"/>
@@ -1553,9 +1577,9 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F41" s="4" t="n"/>
@@ -1579,7 +1603,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1605,7 +1629,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="E43" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1675,7 +1699,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1701,7 +1725,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E47" s="4" t="inlineStr">
+      <c r="E47" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1727,9 +1751,9 @@
           <t>PDF 버전과 GT ITCD 불일치 (버전 미스매치)</t>
         </is>
       </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E48" s="10" t="inlineStr">
+        <is>
+          <t>처리불가</t>
         </is>
       </c>
       <c r="F48" s="8" t="n"/>
@@ -1797,9 +1821,9 @@
           <t>ITCD A02 전용 MAX_AG 상이 — X100/N7/g=1: A01=80 A02=76, X100/N10/g=1: A01=80 A02=71 (PDF 텍스트에 ITCD별 분리 섹션 없음)</t>
         </is>
       </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E51" s="10" t="inlineStr">
+        <is>
+          <t>처리불가</t>
         </is>
       </c>
       <c r="F51" s="8" t="n"/>
@@ -1823,7 +1847,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1849,7 +1873,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr">
+      <c r="E53" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1875,7 +1899,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E54" s="4" t="inlineStr">
+      <c r="E54" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1901,7 +1925,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
+      <c r="E55" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1927,7 +1951,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E56" s="4" t="inlineStr">
+      <c r="E56" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1953,7 +1977,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="E57" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -1979,9 +2003,9 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E58" s="4" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E58" s="9" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F58" s="4" t="n"/>
@@ -2027,9 +2051,9 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E60" s="4" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E60" s="9" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F60" s="4" t="n"/>
@@ -2075,7 +2099,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E62" s="4" t="inlineStr">
+      <c r="E62" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -2101,7 +2125,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E63" s="4" t="inlineStr">
+      <c r="E63" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>
@@ -2149,9 +2173,9 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E65" s="4" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E65" s="9" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F65" s="4" t="n"/>
@@ -2175,9 +2199,9 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E66" s="4" t="inlineStr">
-        <is>
-          <t>미해결</t>
+      <c r="E66" s="9" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F66" s="4" t="n"/>
@@ -2201,7 +2225,7 @@
           <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
         </is>
       </c>
-      <c r="E67" s="4" t="inlineStr">
+      <c r="E67" s="11" t="inlineStr">
         <is>
           <t>미해결</t>
         </is>

</xml_diff>

<commit_message>
Fix 처리불가 logic: respect answer field in structural_issues.xlsx
- ITCD불일치 with answer → '미해결' (implementation possible, path exists)
- ITCD불일치 without answer → '처리불가' (no known solution)
- Changed: 1571, 1726, 1745 처리불가 → 미해결 (all have answers)
- Kept: 2130, 2205 as 처리불가 (no answer written)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/structural_issues.xlsx
+++ b/data/structural_issues.xlsx
@@ -693,9 +693,9 @@
           <t>동일 PDF 내 복수 ITCD 간 보험기간/납입기간 상이</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>처리불가</t>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>미해결</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -953,9 +953,9 @@
           <t>ITCD 039/041 MIN_AG=19, ITCD 040/042 MIN_AG=20 — PDF에 만19세만 존재</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
-        <is>
-          <t>처리불가</t>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>미해결</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -1053,9 +1053,9 @@
           <t>동일 PDF 내 복수 ITCD 간 MIN_AG 상이</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>처리불가</t>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>미해결</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Add annuity onset-offset table extraction + fix 거치형 code conversion
New: _extract_annuity_onset_offset_table (pattern A-0-4) in extraction_rules.py
- Handles "가입최고나이 : 연금개시나이, 납입기간별로 아래와 같음" format
  without [남자]/[여자] blocks (스마트V연금, Wealth직장인연금, 스마트하이브리드연금)
- Parses per-payment-term offset map (N년납/전기납/거치형)
- Supports min_age exception ("단, N종...가입최저나이는 M세")
- Generates max_age < min_age rows per GT convention

Fix: convert_payment_period("") in convert_codes.py
- Empty string → PAYM_TERM_DVSN_CODE="", PAYM_TERM_INQY_CODE="" (거치형)
- Previously returned _convert_error causing batch exit code 1

Result: S00026 PASS 36 → 39 (+1758, +1833, +2042)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/structural_issues.xlsx
+++ b/data/structural_issues.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="맑은 고딕"/>
       <family val="2"/>
@@ -55,8 +55,13 @@
       <sz val="8"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -111,6 +116,11 @@
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -139,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -183,6 +193,11 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -548,11 +563,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -565,27 +580,32 @@
           <t>ISRN_KIND_DTCD</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
+        <is>
+          <t>테이블</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>사업방법서 파일명</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>문제유형</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>문제설명</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>상태</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>답변/해결방법</t>
         </is>
@@ -595,19 +615,19 @@
       <c r="A2" s="2" t="n">
         <v>1224</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>한화생명 기업복지라이프플랜보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E2" s="12" t="inlineStr">
@@ -615,7 +635,12 @@
           <t>해결</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">보기납기 조합이 하나일 경우는 가입나이테이블에 보기납기 정보가 필요없음. </t>
         </is>
@@ -625,19 +650,19 @@
       <c r="A3" s="2" t="n">
         <v>1228</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>한화생명 연금저축 스마트하이드림연금보험_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -645,7 +670,12 @@
           <t>해결</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>나.보험료 납입기간 항목이 납입기간 정보 이다.
 (2) 가입최고나이 : (연금개시나이-납입기간)세  계산하고
@@ -658,71 +688,86 @@
       <c r="A4" s="2" t="n">
         <v>1550</v>
       </c>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n"/>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="n"/>
     </row>
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>1555</v>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n"/>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n"/>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="6" t="n">
         <v>1571</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>한화생명 연금보험Enterprise 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>ITCD불일치</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>동일 PDF 내 복수 ITCD 간 보험기간/납입기간 상이</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>2. 보험기간, 보험료 납입기간, 보험료 납입주기, 피보험자 가입나이 및 연금개시나이 : 보험기간 납입기간 납입주기 연금개시나이 정보가 있는 부분이다.
 나.  보험종목의 구성 이  동일한 ISRN_KIND_DTCD의 ITCD 구분 정보이다. 이 정보를 활용하여 구분 해야 한다.
@@ -734,27 +779,32 @@
       <c r="A7" s="2" t="n">
         <v>1571</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>한화생명 연금보험Enterprise 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>2. 보험기간, 보험료 납입기간, 보험료 납입주기, 피보험자 가입나이 및 연금개시나이 : 보험기간 납입기간 납입주기 연금개시나이 정보가 있는 부분이다.
 나.  보험종목의 구성 이  동일한 ISRN_KIND_DTCD의 ITCD 구분 정보이다. 이 정보를 활용하여 구분 해야 한다.
@@ -766,41 +816,46 @@
       <c r="A8" s="2" t="n">
         <v>1626</v>
       </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="n"/>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="2" t="n">
         <v>1629</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>한화생명 연금저축 미래로기업복지연금보험_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
@@ -808,7 +863,12 @@
           <t>해결</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>2. 보험기간, 보험료 납입기간, 보험료 납입주기, 피보험자 가입나이 및 연금개시나이 : 보험기간 납입기간 납입주기 연금개시나이 정보가 있는 부분이다.
 나.  보험종목의 구성 이  동일한 ISRN_KIND_DTCD의 ITCD 구분 정보이다. 이 정보를 활용하여 구분 해야 한다.
@@ -820,27 +880,32 @@
       <c r="A10" s="6" t="n">
         <v>1629</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>한화생명 연금저축 미래로기업복지연금보험_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>ITCD불일치</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>동일 PDF 내 복수 ITCD 간 보험기간/납입기간 상이</t>
-        </is>
-      </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
           <t>해결</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
         <is>
           <t>2. 보험기간, 보험료 납입기간, 보험료 납입주기, 피보험자 가입나이 및 연금개시나이 : 보험기간 납입기간 납입주기 연금개시나이 정보가 있는 부분이다.
 나.  보험종목의 구성 이  동일한 ISRN_KIND_DTCD의 ITCD 구분 정보이다. 이 정보를 활용하여 구분 해야 한다.
@@ -852,137 +917,167 @@
       <c r="A11" s="2" t="n">
         <v>1651</v>
       </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n"/>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
     </row>
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>1671</v>
       </c>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n"/>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="n"/>
     </row>
     <row r="13" ht="36" customHeight="1">
       <c r="A13" s="2" t="n">
         <v>1700</v>
       </c>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n"/>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="n"/>
     </row>
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>1708</v>
       </c>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n"/>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="n"/>
     </row>
     <row r="15" ht="36" customHeight="1">
       <c r="A15" s="2" t="n">
         <v>1709</v>
       </c>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n"/>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="n"/>
     </row>
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="6" t="n">
         <v>1726</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>한화생명 e정기보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>ITCD불일치</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>ITCD 039/041 MIN_AG=19, ITCD 040/042 MIN_AG=20 — PDF에 만19세만 존재</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
         <is>
           <t>만19세를 19세 인식하게 해줘
 표준체/건강체 분리상품의 경우 건강체 가입조건은 표준체 조건을 준용하되, 가입가능 최저나이가 20세 미만일 경우에 한하여 20세로 치환</t>
@@ -993,97 +1088,117 @@
       <c r="A17" s="2" t="n">
         <v>1736</v>
       </c>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n"/>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="n"/>
     </row>
     <row r="18" ht="36" customHeight="1">
       <c r="A18" s="2" t="n">
         <v>1743</v>
       </c>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n"/>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="n"/>
     </row>
     <row r="19" ht="36" customHeight="1">
       <c r="A19" s="2" t="n">
         <v>1745</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>한화생명 연금저축 하이드림연금보험_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E19" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="n"/>
     </row>
     <row r="20" ht="36" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>1745</v>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>한화생명 연금저축 하이드림연금보험_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>ITCD불일치</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>동일 PDF 내 복수 ITCD 간 MIN_AG 상이</t>
-        </is>
-      </c>
-      <c r="E20" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
         <is>
           <t>1. 보험종목에 관한 사항
 나.  보험종목의 구성 이  동일한 ISRN_KIND_DTCD의 ITCD 구분 정보이다. 이 정보를 활용하여 구분 해야 한다.
@@ -1095,229 +1210,274 @@
       <c r="A21" s="2" t="n">
         <v>1752</v>
       </c>
-      <c r="B21" s="5" t="n"/>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n"/>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="n"/>
     </row>
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="2" t="n">
         <v>1753</v>
       </c>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="n"/>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="n"/>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="2" t="n">
         <v>1758</v>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>한화생명 스마트V연금보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E23" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="n"/>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="2" t="n">
         <v>1760</v>
       </c>
-      <c r="B24" s="5" t="n"/>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="n"/>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="n"/>
     </row>
     <row r="25" ht="36" customHeight="1">
       <c r="A25" s="2" t="n">
         <v>1764</v>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>한화생명 H 기업재해보장보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E25" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="n"/>
     </row>
     <row r="26" ht="36" customHeight="1">
       <c r="A26" s="2" t="n">
         <v>1772</v>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>한화생명 e연금저축보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E26" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="n"/>
     </row>
     <row r="27" ht="36" customHeight="1">
       <c r="A27" s="2" t="n">
         <v>1781</v>
       </c>
-      <c r="B27" s="5" t="n"/>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n"/>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="n"/>
     </row>
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="2" t="n">
         <v>1789</v>
       </c>
-      <c r="B28" s="5" t="n"/>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="n"/>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="n"/>
     </row>
     <row r="29" ht="36" customHeight="1">
       <c r="A29" s="2" t="n">
         <v>1795</v>
       </c>
-      <c r="B29" s="5" t="n"/>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="n"/>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="n"/>
     </row>
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="2" t="n">
         <v>1808</v>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>한화생명 노후실손의료비보장보험(갱신형) 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -1325,99 +1485,119 @@
           <t>해결</t>
         </is>
       </c>
-      <c r="F30" s="4" t="n"/>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="n"/>
     </row>
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="2" t="n">
         <v>1809</v>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>한화생명 연금저축 미래로기업복지연금보험_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E31" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="n"/>
     </row>
     <row r="32" ht="36" customHeight="1">
       <c r="A32" s="2" t="n">
         <v>1833</v>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>한화생명 Wealth직장인연금보험 무배당_사업방법서_20260130~.pdf</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E32" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="n"/>
     </row>
     <row r="33" ht="36" customHeight="1">
       <c r="A33" s="2" t="n">
         <v>1845</v>
       </c>
-      <c r="B33" s="5" t="n"/>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="n"/>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="n"/>
     </row>
     <row r="34" ht="36" customHeight="1">
       <c r="A34" s="2" t="n">
         <v>1946</v>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>한화생명 노후실손의료비보장보험(갱신형) 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -1425,25 +1605,30 @@
           <t>해결</t>
         </is>
       </c>
-      <c r="F34" s="4" t="n"/>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="n"/>
     </row>
     <row r="35" ht="36" customHeight="1">
       <c r="A35" s="2" t="n">
         <v>1950</v>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>한화생명 튼튼이 치아보험(갱신형) 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E35" s="12" t="inlineStr">
@@ -1451,25 +1636,30 @@
           <t>해결</t>
         </is>
       </c>
-      <c r="F35" s="4" t="n"/>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="n"/>
     </row>
     <row r="36" ht="36" customHeight="1">
       <c r="A36" s="2" t="n">
         <v>1976</v>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>한화생명 간편가입 실손의료비보장보험(갱신형) 무배당(재가입용)_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
@@ -1477,103 +1667,123 @@
           <t>해결</t>
         </is>
       </c>
-      <c r="F36" s="4" t="n"/>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="n"/>
     </row>
     <row r="37" ht="36" customHeight="1">
       <c r="A37" s="2" t="n">
         <v>1982</v>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>한화생명 기본형 급여 실손의료비보장보험(갱신형) 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E37" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F37" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="n"/>
     </row>
     <row r="38" ht="36" customHeight="1">
       <c r="A38" s="2" t="n">
         <v>1983</v>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>한화생명 기본형 급여 e실손의료비보장보험(갱신형) 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E38" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E38" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="n"/>
     </row>
     <row r="39" ht="36" customHeight="1">
       <c r="A39" s="2" t="n">
         <v>1984</v>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>한화생명 기본형 급여 실손의료비보장보험(계약전환 단체개인전환 개인중지재개용)(갱신형) 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E39" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="n"/>
     </row>
     <row r="40" ht="36" customHeight="1">
       <c r="A40" s="2" t="n">
         <v>1985</v>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>한화생명 기본형 급여 실손의료비보장보험(계약전환 단체개인전환 개인중지재개용)(갱신형) 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -1581,25 +1791,30 @@
           <t>해결</t>
         </is>
       </c>
-      <c r="F40" s="4" t="n"/>
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="n"/>
     </row>
     <row r="41" ht="36" customHeight="1">
       <c r="A41" s="2" t="n">
         <v>1986</v>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>한화생명 기본형 급여 실손의료비보장보험(계약전환 단체개인전환 개인중지재개용)(갱신형) 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E41" s="12" t="inlineStr">
@@ -1607,425 +1822,510 @@
           <t>해결</t>
         </is>
       </c>
-      <c r="F41" s="4" t="n"/>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="n"/>
     </row>
     <row r="42" ht="36" customHeight="1">
       <c r="A42" s="2" t="n">
         <v>2042</v>
       </c>
-      <c r="B42" s="3" t="inlineStr">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
         <is>
           <t>한화생명 스마트하이브리드연금보험 무배당_사업방법서_20260201~.pdf</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E42" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E42" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F42" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="n"/>
     </row>
     <row r="43" ht="36" customHeight="1">
       <c r="A43" s="2" t="n">
         <v>2126</v>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
         <is>
           <t>한화생명 상생친구 보장보험 무배당_사업방법서_20260201~.pdf</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E43" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F43" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="n"/>
     </row>
     <row r="44" ht="36" customHeight="1">
       <c r="A44" s="2" t="n">
         <v>2127</v>
       </c>
-      <c r="B44" s="5" t="n"/>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="n"/>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="n"/>
     </row>
     <row r="45" ht="36" customHeight="1">
       <c r="A45" s="2" t="n">
         <v>2128</v>
       </c>
-      <c r="B45" s="5" t="n"/>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="n"/>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="n"/>
     </row>
     <row r="46" ht="36" customHeight="1">
       <c r="A46" s="2" t="n">
         <v>2129</v>
       </c>
-      <c r="B46" s="3" t="inlineStr">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
         <is>
           <t>한화생명 상속H종신보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E46" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F46" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="n"/>
     </row>
     <row r="47" ht="36" customHeight="1">
       <c r="A47" s="2" t="n">
         <v>2130</v>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
         <is>
           <t>한화생명 간편가입 상속H종신보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E47" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F47" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="n"/>
     </row>
     <row r="48" ht="36" customHeight="1">
       <c r="A48" s="6" t="n">
         <v>2130</v>
       </c>
-      <c r="B48" s="7" t="inlineStr">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
         <is>
           <t>한화생명 간편가입 상속H종신보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C48" s="8" t="inlineStr">
+      <c r="D48" s="8" t="inlineStr">
         <is>
           <t>ITCD불일치</t>
         </is>
       </c>
-      <c r="D48" s="8" t="inlineStr">
+      <c r="E48" s="8" t="inlineStr">
         <is>
           <t>PDF 버전과 GT ITCD 불일치 (버전 미스매치)</t>
         </is>
       </c>
-      <c r="E48" s="14" t="inlineStr">
+      <c r="F48" s="14" t="inlineStr">
         <is>
           <t>처리불가</t>
         </is>
       </c>
-      <c r="F48" s="8" t="n"/>
+      <c r="G48" s="8" t="n"/>
     </row>
     <row r="49" ht="36" customHeight="1">
       <c r="A49" s="2" t="n">
         <v>2172</v>
       </c>
-      <c r="B49" s="5" t="n"/>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="n"/>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="n"/>
     </row>
     <row r="50" ht="36" customHeight="1">
       <c r="A50" s="2" t="n">
         <v>2174</v>
       </c>
-      <c r="B50" s="5" t="n"/>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="n"/>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F50" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="n"/>
     </row>
     <row r="51" ht="36" customHeight="1">
       <c r="A51" s="6" t="n">
         <v>2205</v>
       </c>
-      <c r="B51" s="7" t="inlineStr">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
         <is>
           <t>한화생명 간편가입 시그니처H보장보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C51" s="8" t="inlineStr">
+      <c r="D51" s="8" t="inlineStr">
         <is>
           <t>ITCD불일치</t>
         </is>
       </c>
-      <c r="D51" s="8" t="inlineStr">
+      <c r="E51" s="8" t="inlineStr">
         <is>
           <t>ITCD A02 전용 MAX_AG 상이 — X100/N7/g=1: A01=80 A02=76, X100/N10/g=1: A01=80 A02=71 (PDF 텍스트에 ITCD별 분리 섹션 없음)</t>
         </is>
       </c>
-      <c r="E51" s="14" t="inlineStr">
+      <c r="F51" s="14" t="inlineStr">
         <is>
           <t>처리불가</t>
         </is>
       </c>
-      <c r="F51" s="8" t="n"/>
+      <c r="G51" s="8" t="n"/>
     </row>
     <row r="52" ht="36" customHeight="1">
       <c r="A52" s="2" t="n">
         <v>2207</v>
       </c>
-      <c r="B52" s="3" t="inlineStr">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
         <is>
           <t>한화생명 제로백H종신보험 무배당_사업방법서_20260201~.pdf</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E52" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F52" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="n"/>
     </row>
     <row r="53" ht="36" customHeight="1">
       <c r="A53" s="2" t="n">
         <v>2208</v>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
         <is>
           <t>한화생명 간편가입 제로백H종신보험 무배당_사업방법서_20260201~.pdf</t>
         </is>
       </c>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E53" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F53" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="n"/>
     </row>
     <row r="54" ht="36" customHeight="1">
       <c r="A54" s="2" t="n">
         <v>2209</v>
       </c>
-      <c r="B54" s="3" t="inlineStr">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
         <is>
           <t>한화생명 H종신보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E54" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F54" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F54" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="n"/>
     </row>
     <row r="55" ht="36" customHeight="1">
       <c r="A55" s="2" t="n">
         <v>2210</v>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
         <is>
           <t>한화생명 간편가입 H종신보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E55" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F55" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="n"/>
     </row>
     <row r="56" ht="36" customHeight="1">
       <c r="A56" s="2" t="n">
         <v>2242</v>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
         <is>
           <t>한화생명 경영인H정기보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E56" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F56" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="n"/>
     </row>
     <row r="57" ht="36" customHeight="1">
       <c r="A57" s="2" t="n">
         <v>2243</v>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>한화생명 간편가입 경영인H정기보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E57" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F57" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="n"/>
     </row>
     <row r="58" ht="36" customHeight="1">
       <c r="A58" s="2" t="n">
         <v>2244</v>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>한화생명 케어백간병플러스보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -2033,47 +2333,57 @@
           <t>해결</t>
         </is>
       </c>
-      <c r="F58" s="4" t="n"/>
+      <c r="F58" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="n"/>
     </row>
     <row r="59" ht="36" customHeight="1">
       <c r="A59" s="2" t="n">
         <v>2245</v>
       </c>
-      <c r="B59" s="5" t="n"/>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="n"/>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F59" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="n"/>
     </row>
     <row r="60" ht="36" customHeight="1">
       <c r="A60" s="2" t="n">
         <v>2246</v>
       </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
         <is>
           <t>한화생명 H건강플러스보험 무배당_사업방법서_20260201~.pdf</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E60" s="12" t="inlineStr">
@@ -2081,121 +2391,146 @@
           <t>해결</t>
         </is>
       </c>
-      <c r="F60" s="4" t="n"/>
+      <c r="F60" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="n"/>
     </row>
     <row r="61" ht="36" customHeight="1">
       <c r="A61" s="2" t="n">
         <v>2247</v>
       </c>
-      <c r="B61" s="5" t="n"/>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="n"/>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F61" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="n"/>
     </row>
     <row r="62" ht="36" customHeight="1">
       <c r="A62" s="2" t="n">
         <v>2250</v>
       </c>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
         <is>
           <t>한화생명 하나로H종신보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E62" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F62" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F62" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="n"/>
     </row>
     <row r="63" ht="36" customHeight="1">
       <c r="A63" s="2" t="n">
         <v>2251</v>
       </c>
-      <c r="B63" s="3" t="inlineStr">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
         <is>
           <t>한화생명 간편가입 하나로H종신보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C63" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E63" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F63" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F63" s="13" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="n"/>
     </row>
     <row r="64" ht="36" customHeight="1">
       <c r="A64" s="2" t="n">
         <v>2252</v>
       </c>
-      <c r="B64" s="5" t="n"/>
-      <c r="C64" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="n"/>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F64" s="4" t="n"/>
+          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="n"/>
     </row>
     <row r="65" ht="36" customHeight="1">
       <c r="A65" s="2" t="n">
         <v>2255</v>
       </c>
-      <c r="B65" s="3" t="inlineStr">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
         <is>
           <t>한화생명 포켓골절보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C65" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E65" s="12" t="inlineStr">
@@ -2203,25 +2538,30 @@
           <t>해결</t>
         </is>
       </c>
-      <c r="F65" s="4" t="n"/>
+      <c r="F65" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="n"/>
     </row>
     <row r="66" ht="36" customHeight="1">
       <c r="A66" s="2" t="n">
         <v>2256</v>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
         <is>
           <t>한화생명 간편가입 포켓골절보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C66" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+          <t>GT_NaN</t>
         </is>
       </c>
       <c r="E66" s="12" t="inlineStr">
@@ -2229,33 +2569,193 @@
           <t>해결</t>
         </is>
       </c>
-      <c r="F66" s="4" t="n"/>
+      <c r="F66" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="n"/>
     </row>
     <row r="67" ht="36" customHeight="1">
       <c r="A67" s="2" t="n">
         <v>2259</v>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>S00026</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
         <is>
           <t>한화생명 바로연금보험 무배당_사업방법서_20260101~.pdf</t>
         </is>
       </c>
-      <c r="C67" s="4" t="inlineStr">
-        <is>
-          <t>GT_NaN</t>
-        </is>
-      </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
-        </is>
-      </c>
-      <c r="E67" s="13" t="inlineStr">
-        <is>
-          <t>미해결</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="n"/>
+          <t>GT_NaN</t>
+        </is>
+      </c>
+      <c r="E67" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F67" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>1629</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>S00027</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>미래로기업복지연금보험</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>확정기간연금_onset_range</t>
+        </is>
+      </c>
+      <c r="E68" s="17" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F68" s="16" t="inlineStr">
+        <is>
+          <t>처리불가</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>1745</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>S00027</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>스마트하이드림연금보험</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>확정기간연금_onset_range</t>
+        </is>
+      </c>
+      <c r="E69" s="17" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F69" s="16" t="inlineStr">
+        <is>
+          <t>처리불가</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>1772</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>S00027</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>e연금저축보험</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>확정기간연금_N년형없음</t>
+        </is>
+      </c>
+      <c r="E70" s="17" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F70" s="16" t="inlineStr">
+        <is>
+          <t>처리불가</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>1809</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>S00027</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>미래로기업복지연금보험</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>확정기간연금_onset_range</t>
+        </is>
+      </c>
+      <c r="E71" s="17" t="inlineStr">
+        <is>
+          <t>해결</t>
+        </is>
+      </c>
+      <c r="F71" s="16" t="inlineStr">
+        <is>
+          <t>처리불가</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>2126</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>S00027</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>상생친구보험/진심가득보험</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>ITCD부재</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>갱신형 1년만기 X1 ITCD: PDF 내 해당 ITCD 정보 없음, X1/N0 행 생성 불가</t>
+        </is>
+      </c>
+      <c r="F72" s="16" t="inlineStr">
+        <is>
+          <t>처리불가</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Improve S00026 일치율 39→46: 키셋 비교 복구, PROD_ITCD 필터, cross-page 테이블 처리
세션16 주요 변경:
- generate_report.py: raw count → 키셋 비교(miss_cnt==0), S00026 결과 PASS/FAIL→일치/불일치, itcd_pairs 필터, 불일치사유 컬럼
- model_key_loader.py: get_active_key_cols GT-only→GT AND EX 교집합(#3f8248f 버그 복구)
- extraction_rules.py: _parse_age_table_separate_minmax에 cross-page 테이블 분할 처리 추가(2210 일치)
- update_structural_issues.py: PASS/FAIL→일치/불일치 기준 업데이트
- structural_issues.xlsx: 7개 DTCD 해결 처리(2205/A01, 2207~2210, 2250, 2251)
- CLAUDE.md: 결과코드 문서 업데이트

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/structural_issues.xlsx
+++ b/data/structural_issues.xlsx
@@ -2111,9 +2111,9 @@
           <t>ITCD불일치</t>
         </is>
       </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>ITCD A02 전용 MAX_AG 상이 — X100/N7/g=1: A01=80 A02=76, X100/N10/g=1: A01=80 A02=71 (PDF 텍스트에 ITCD별 분리 섹션 없음)</t>
+      <c r="E51" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F51" s="14" t="inlineStr">
@@ -2142,9 +2142,9 @@
           <t>GT_NaN</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
-        <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+      <c r="E52" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F52" s="13" t="inlineStr">
@@ -2173,9 +2173,9 @@
           <t>GT_NaN</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr">
-        <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+      <c r="E53" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F53" s="13" t="inlineStr">
@@ -2204,9 +2204,9 @@
           <t>GT_NaN</t>
         </is>
       </c>
-      <c r="E54" s="4" t="inlineStr">
-        <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+      <c r="E54" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F54" s="13" t="inlineStr">
@@ -2235,9 +2235,9 @@
           <t>GT_NaN</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+      <c r="E55" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F55" s="13" t="inlineStr">
@@ -2444,9 +2444,9 @@
           <t>GT_NaN</t>
         </is>
       </c>
-      <c r="E62" s="4" t="inlineStr">
-        <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+      <c r="E62" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F62" s="13" t="inlineStr">
@@ -2475,9 +2475,9 @@
           <t>GT_NaN</t>
         </is>
       </c>
-      <c r="E63" s="4" t="inlineStr">
-        <is>
-          <t>GT 데이터에 ISRN_TERM_DVSN_CODE 또는 PAYM_TERM_DVSN_CODE가 NaN — 키 비교 불가</t>
+      <c r="E63" s="12" t="inlineStr">
+        <is>
+          <t>해결</t>
         </is>
       </c>
       <c r="F63" s="13" t="inlineStr">

</xml_diff>